<commit_message>
First draft for #781
</commit_message>
<xml_diff>
--- a/jeaf-generator-test-deprecation-report/src-gen/main/resources/Breaking_Changes.xlsx
+++ b/jeaf-generator-test-deprecation-report/src-gen/main/resources/Breaking_Changes.xlsx
@@ -251,7 +251,7 @@
     <t>7.0</t>
   </si>
   <si>
-    <t>2026-09-13</t>
+    <t>2026-12-24</t>
   </si>
   <si>
     <t>upcomingMandatoryProperty</t>
@@ -272,7 +272,7 @@
     <t>8.0</t>
   </si>
   <si>
-    <t>2026-10-20</t>
+    <t>2027-05-01</t>
   </si>
 </sst>
 </file>

</xml_diff>